<commit_message>
n8n board refresh 2026-07-08T17:38:52Z
</commit_message>
<xml_diff>
--- a/app/reports/HDRN_research.xlsx
+++ b/app/reports/HDRN_research.xlsx
@@ -617,7 +617,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-07 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-08 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>2.035</v>
+        <v>1.9626</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -852,7 +852,7 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>0.04525000095367432</v>
+        <v>0.04577000141143799</v>
       </c>
     </row>
     <row r="6">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="B35" s="18" t="n">
-        <v>71498842.26044226</v>
+        <v>71498836.23764394</v>
       </c>
     </row>
     <row r="36">
@@ -1202,7 +1202,7 @@
         </is>
       </c>
       <c r="B37" s="20" t="n">
-        <v>2.035</v>
+        <v>1.9626</v>
       </c>
     </row>
     <row r="38">
@@ -1481,7 +1481,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>145500144</v>
+        <v>140323616</v>
       </c>
       <c r="D5" s="29" t="n"/>
       <c r="E5" s="29" t="n">
@@ -1581,7 +1581,7 @@
         </is>
       </c>
       <c r="C10" s="30" t="n">
-        <v>387750016</v>
+        <v>388500000</v>
       </c>
       <c r="D10" s="31" t="n"/>
       <c r="E10" s="31" t="n"/>
@@ -1599,10 +1599,10 @@
         </is>
       </c>
       <c r="C11" s="30" t="n">
-        <v>359835008</v>
+        <v>359490016</v>
       </c>
       <c r="D11" s="31" t="n">
-        <v>32.59375</v>
+        <v>32.5625</v>
       </c>
       <c r="E11" s="31" t="n"/>
       <c r="F11" s="31" t="n"/>
@@ -1619,10 +1619,10 @@
         </is>
       </c>
       <c r="C12" s="30" t="n">
-        <v>395447648</v>
+        <v>393946880</v>
       </c>
       <c r="D12" s="31" t="n">
-        <v>30.114286</v>
+        <v>30</v>
       </c>
       <c r="E12" s="31" t="n"/>
       <c r="F12" s="31" t="n"/>

</xml_diff>